<commit_message>
chore: rename pricing files, update task-management + Notion CSV
- Rename: 09_成果報酬3%説明シート.md → 09_成約報酬50万円説明シート.md
- Rename: 10_成果報酬3%契約別紙.md → 10_成約報酬契約別紙.md
- task-management.xlsx: add 8 pricing model change tasks (PR-001~PR-008)
  across dashboard, PM, sales, and legal sheets
- Notion CSV: append 8 pricing tasks (105 total)
- Final scan: zero remaining "成果報酬3%" references in md/code

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/最新版/02_管理シート/task-management.xlsx
+++ b/docs/最新版/02_管理シート/task-management.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5963,9 +5963,463 @@
         </is>
       </c>
     </row>
+    <row r="110" ht="24" customHeight="1">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>■ 料金モデル変更対応 (成約報酬50万円) (8件)</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="n"/>
+      <c r="C110" s="9" t="n"/>
+      <c r="D110" s="9" t="n"/>
+      <c r="E110" s="9" t="n"/>
+      <c r="F110" s="9" t="n"/>
+      <c r="G110" s="9" t="n"/>
+      <c r="H110" s="9" t="n"/>
+      <c r="I110" s="9" t="n"/>
+      <c r="J110" s="9" t="n"/>
+      <c r="K110" s="9" t="n"/>
+      <c r="L110" s="10" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="11" t="inlineStr">
+        <is>
+          <t>PR-001</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>旧3%記述→50万円: 全md資料更新完了</t>
+        </is>
+      </c>
+      <c r="C111" s="11" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D111" s="11" t="inlineStr">
+        <is>
+          <t>PM進行管理</t>
+        </is>
+      </c>
+      <c r="E111" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F111" s="11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="G111" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="H111" s="11" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="I111" s="11" t="inlineStr"/>
+      <c r="J111" s="11" t="inlineStr"/>
+      <c r="K111" s="11" t="inlineStr">
+        <is>
+          <t>21ファイル更新済み</t>
+        </is>
+      </c>
+      <c r="L111" s="11" t="inlineStr">
+        <is>
+          <t>dfa8d73</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="inlineStr">
+        <is>
+          <t>PR-002</t>
+        </is>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>旧3%記述→50万円: コード(FixedBar.tsx)更新</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D112" s="11" t="inlineStr">
+        <is>
+          <t>開発</t>
+        </is>
+      </c>
+      <c r="E112" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F112" s="11" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="G112" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="H112" s="11" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="I112" s="11" t="inlineStr"/>
+      <c r="J112" s="11" t="inlineStr"/>
+      <c r="K112" s="11" t="inlineStr">
+        <is>
+          <t>コメント2箇所修正</t>
+        </is>
+      </c>
+      <c r="L112" s="11" t="inlineStr">
+        <is>
+          <t>dfa8d73</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="11" t="inlineStr">
+        <is>
+          <t>PR-003</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>旧3%記述→50万円: ファイルリネーム(09_/10_)</t>
+        </is>
+      </c>
+      <c r="C113" s="11" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D113" s="11" t="inlineStr">
+        <is>
+          <t>PM進行管理</t>
+        </is>
+      </c>
+      <c r="E113" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F113" s="11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="G113" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="H113" s="11" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="I113" s="11" t="inlineStr"/>
+      <c r="J113" s="11" t="inlineStr"/>
+      <c r="K113" s="11" t="inlineStr">
+        <is>
+          <t>git mv完了</t>
+        </is>
+      </c>
+      <c r="L113" s="11" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="inlineStr">
+        <is>
+          <t>PR-004</t>
+        </is>
+      </c>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>docx/pptx/xlsx内の旧料金記述を差し替え原稿で更新</t>
+        </is>
+      </c>
+      <c r="C114" s="11" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="inlineStr">
+        <is>
+          <t>PM進行管理</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F114" s="11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="G114" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="H114" s="11" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="I114" s="11" t="inlineStr"/>
+      <c r="J114" s="11" t="inlineStr"/>
+      <c r="K114" s="11" t="inlineStr">
+        <is>
+          <t>03_営業/04_経理/05_契約/06_戦略/07_運用のdocx更新</t>
+        </is>
+      </c>
+      <c r="L114" s="11" t="inlineStr">
+        <is>
+          <t>md最新版を正として差替</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="inlineStr">
+        <is>
+          <t>PR-005</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>契約別紙(50万円版)を弁護士に送付</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D115" s="11" t="inlineStr">
+        <is>
+          <t>契約法務</t>
+        </is>
+      </c>
+      <c r="E115" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F115" s="11" t="inlineStr">
+        <is>
+          <t>代表</t>
+        </is>
+      </c>
+      <c r="G115" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="H115" s="11" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="I115" s="11" t="inlineStr"/>
+      <c r="J115" s="11" t="inlineStr">
+        <is>
+          <t>PR-001</t>
+        </is>
+      </c>
+      <c r="K115" s="11" t="inlineStr">
+        <is>
+          <t>弁護士にメール送信</t>
+        </is>
+      </c>
+      <c r="L115" s="11" t="inlineStr">
+        <is>
+          <t>L-001/L-002と同時</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="12" t="inlineStr">
+        <is>
+          <t>PR-006</t>
+        </is>
+      </c>
+      <c r="B116" s="12" t="inlineStr">
+        <is>
+          <t>営業向け50万円モデル説明会実施</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D116" s="12" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="E116" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="G116" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="H116" s="12" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="I116" s="12" t="inlineStr"/>
+      <c r="J116" s="12" t="inlineStr">
+        <is>
+          <t>PR-004</t>
+        </is>
+      </c>
+      <c r="K116" s="12" t="inlineStr">
+        <is>
+          <t>営業全員が50万円の説明可能</t>
+        </is>
+      </c>
+      <c r="L116" s="12" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="12" t="inlineStr">
+        <is>
+          <t>PR-007</t>
+        </is>
+      </c>
+      <c r="B117" s="12" t="inlineStr">
+        <is>
+          <t>成約報酬対象判定フロー図を社内共有</t>
+        </is>
+      </c>
+      <c r="C117" s="12" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D117" s="12" t="inlineStr">
+        <is>
+          <t>PM進行管理</t>
+        </is>
+      </c>
+      <c r="E117" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F117" s="12" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="G117" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="H117" s="12" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="I117" s="12" t="inlineStr"/>
+      <c r="J117" s="12" t="inlineStr">
+        <is>
+          <t>PR-001</t>
+        </is>
+      </c>
+      <c r="K117" s="12" t="inlineStr">
+        <is>
+          <t>判定フロー図をSlack共有</t>
+        </is>
+      </c>
+      <c r="L117" s="12" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="inlineStr">
+        <is>
+          <t>PR-008</t>
+        </is>
+      </c>
+      <c r="B118" s="12" t="inlineStr">
+        <is>
+          <t>工務店10社に50万円モデル事前説明</t>
+        </is>
+      </c>
+      <c r="C118" s="12" t="inlineStr">
+        <is>
+          <t>Phase0</t>
+        </is>
+      </c>
+      <c r="D118" s="12" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="E118" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="G118" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="H118" s="12" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="I118" s="12" t="inlineStr"/>
+      <c r="J118" s="12" t="inlineStr">
+        <is>
+          <t>PR-006</t>
+        </is>
+      </c>
+      <c r="K118" s="12" t="inlineStr">
+        <is>
+          <t>全10社に説明完了</t>
+        </is>
+      </c>
+      <c r="L118" s="12" t="inlineStr">
+        <is>
+          <t>Phase3開始前告知</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A5:L110"/>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A78:L78"/>
     <mergeCell ref="A101:L101"/>
     <mergeCell ref="A2:L2"/>
@@ -5977,6 +6431,7 @@
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="A6:L6"/>
     <mergeCell ref="A56:L56"/>
+    <mergeCell ref="A110:L110"/>
     <mergeCell ref="A67:L67"/>
     <mergeCell ref="J3:L3"/>
   </mergeCells>
@@ -13008,7 +13463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13643,13 +14098,197 @@
       <c r="H20" s="13" t="inlineStr"/>
       <c r="I20" s="13" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>■ 料金モデル変更対応</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n"/>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9" t="n"/>
+      <c r="I21" s="10" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>PR-001</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>旧3%記述→50万円: 全md資料更新完了</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>21ファイル更新済み</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr"/>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>dfa8d73</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>PR-003</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>旧3%記述→50万円: ファイルリネーム(09_/10_)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>git mv完了</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr"/>
+      <c r="I23" s="11" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>PR-004</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>docx/pptx/xlsx内の旧料金記述を差し替え原稿で更新</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>03_営業/04_経理/05_契約/06_戦略/07_運用のdocx更新</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr"/>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>md最新版を正として差替</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>PR-007</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>成約報酬対象判定フロー図を社内共有</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>判定フロー図をSlack共有</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>PR-001</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A18:I18"/>
     <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A21:I21"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13662,7 +14301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14049,10 +14688,116 @@
       <c r="H12" s="13" t="inlineStr"/>
       <c r="I12" s="13" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>■ 料金モデル変更対応</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>PR-006</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>営業向け50万円モデル説明会実施</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>営業全員が50万円の説明可能</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>PR-004</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>PR-008</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>工務店10社に50万円モデル事前説明</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>全10社に説明完了</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>PR-006</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Phase3開始前告知</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A13:I13"/>
     <mergeCell ref="A11:I11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15185,7 +15930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15537,9 +16282,72 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>■ 料金モデル変更対応</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>PR-005</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>契約別紙(50万円版)を弁護士に送付</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>代表</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>弁護士にメール送信</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>PR-001</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>L-001/L-002と同時</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A12:I12"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A10:I10"/>
   </mergeCells>

</xml_diff>